<commit_message>
Update the reference results files after changing pdmake to use the settings tab for checking accuracy
</commit_message>
<xml_diff>
--- a/Examples/Experiment/AlN/results.ref.xlsx
+++ b/Examples/Experiment/AlN/results.ref.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="131">
   <si>
     <t>Directory</t>
   </si>
@@ -46,9 +46,6 @@
   </si>
   <si>
     <t>AlN.exp</t>
-  </si>
-  <si>
-    <t>Phonopy QM program</t>
   </si>
   <si>
     <t>Program</t>
@@ -102,7 +99,22 @@
     <t>Optical permittivity edited</t>
   </si>
   <si>
+    <t>Raman activity units</t>
+  </si>
+  <si>
+    <t>polarizability</t>
+  </si>
+  <si>
     <t>Sigma value</t>
+  </si>
+  <si>
+    <t>Spectroscopy type</t>
+  </si>
+  <si>
+    <t>Powder Infrared</t>
+  </si>
+  <si>
+    <t>Symmetrise optical permittivity</t>
   </si>
   <si>
     <t>Mode</t>
@@ -117,13 +129,22 @@
     <t>Frequency(cm-1)</t>
   </si>
   <si>
-    <t>Intensity(Debye2/Angs2/amu</t>
+    <t>Intensity(Debye2/Angs2/amu)</t>
   </si>
   <si>
-    <t>Integrated Molar Absorption(/L/mole/cm2</t>
+    <t>Integrated Molar Absorption(L/mole/cm2)</t>
   </si>
   <si>
     <t>Absorption maximum (L/mole/cm)</t>
+  </si>
+  <si>
+    <t>Raman R_total (Å⁴/amu)</t>
+  </si>
+  <si>
+    <t>Raman R_parallel (Å⁴/amu)</t>
+  </si>
+  <si>
+    <t>Raman R_perp (Å⁴/amu)</t>
   </si>
   <si>
     <t>No</t>
@@ -153,6 +174,36 @@
     <t>Angle of incidence</t>
   </si>
   <si>
+    <t>Approximate ES</t>
+  </si>
+  <si>
+    <t>Azimuthal sweep points</t>
+  </si>
+  <si>
+    <t>Coalesce equivalent layers</t>
+  </si>
+  <si>
+    <t>Collection angle</t>
+  </si>
+  <si>
+    <t>Collection side</t>
+  </si>
+  <si>
+    <t>superstrate</t>
+  </si>
+  <si>
+    <t>Depth coherence</t>
+  </si>
+  <si>
+    <t>Coherent amplitude</t>
+  </si>
+  <si>
+    <t>Detected polarisation</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
     <t>Filter kernel size</t>
   </si>
   <si>
@@ -165,10 +216,25 @@
     <t>wavenumber</t>
   </si>
   <si>
+    <t>GL point density</t>
+  </si>
+  <si>
     <t>Global azimuthal angle</t>
   </si>
   <si>
+    <t>Incident polarisation</t>
+  </si>
+  <si>
+    <t>Laser wavelength nm</t>
+  </si>
+  <si>
     <t>Layer azimuthals</t>
+  </si>
+  <si>
+    <t>Layer combination</t>
+  </si>
+  <si>
+    <t>Incoherent intensities</t>
   </si>
   <si>
     <t>Layer dielectric flags</t>
@@ -195,6 +261,12 @@
     <t>6H-SiC</t>
   </si>
   <si>
+    <t>Layer NAC mode</t>
+  </si>
+  <si>
+    <t>geometry</t>
+  </si>
+  <si>
     <t>Layer thickness units</t>
   </si>
   <si>
@@ -219,6 +291,24 @@
     <t>DataBase.xlsx</t>
   </si>
   <si>
+    <t>Modal pair combination</t>
+  </si>
+  <si>
+    <t>Group q channels</t>
+  </si>
+  <si>
+    <t>Modal pair final-state model</t>
+  </si>
+  <si>
+    <t>Bulk phase matched</t>
+  </si>
+  <si>
+    <t>Modal pair include zero q</t>
+  </si>
+  <si>
+    <t>Modal pair q-angle tolerance</t>
+  </si>
+  <si>
     <t>Transfer matrix</t>
   </si>
   <si>
@@ -234,16 +324,25 @@
     <t>Percentage partial incoherence</t>
   </si>
   <si>
+    <t>Porto notation</t>
+  </si>
+  <si>
+    <t>Raman electro-optic term</t>
+  </si>
+  <si>
     <t>Scenario type</t>
   </si>
   <si>
-    <t>Single crystal</t>
+    <t>Crystal Infrared</t>
   </si>
   <si>
     <t>Slice thickness</t>
   </si>
   <si>
     <t>Slice thickness unit</t>
+  </si>
+  <si>
+    <t>Temperature K</t>
   </si>
   <si>
     <t>D</t>
@@ -650,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -698,15 +797,15 @@
       <c r="B5" t="s">
         <v>7</v>
       </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
         <v>9</v>
       </c>
     </row>
@@ -717,21 +816,24 @@
       <c r="B7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C7" t="s">
         <v>11</v>
       </c>
-      <c r="C8" t="s">
+    </row>
+    <row r="9" spans="1:3">
+      <c r="B9" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="B10" t="s">
-        <v>13</v>
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -739,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -750,7 +852,7 @@
         <v>1</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -761,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -772,7 +874,7 @@
         <v>1</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -783,7 +885,7 @@
         <v>1</v>
       </c>
       <c r="B15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -794,7 +896,7 @@
         <v>1</v>
       </c>
       <c r="B16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -805,7 +907,7 @@
         <v>1</v>
       </c>
       <c r="B17">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -816,7 +918,7 @@
         <v>1</v>
       </c>
       <c r="B18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -827,7 +929,7 @@
         <v>1</v>
       </c>
       <c r="B19">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -838,7 +940,7 @@
         <v>1</v>
       </c>
       <c r="B20">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -849,20 +951,9 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22">
-        <v>1</v>
-      </c>
-      <c r="B22">
-        <v>11</v>
-      </c>
-      <c r="C22">
         <v>0</v>
       </c>
     </row>
@@ -878,13 +969,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3713,25 +3804,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="B1" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="D1" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="E1" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="F1" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="G1" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="H1" t="s">
-        <v>97</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -8972,25 +9063,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="B1" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="D1" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="E1" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="F1" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="G1" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="H1" t="s">
-        <v>97</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -14226,12 +14317,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="B1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -14239,7 +14330,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -14250,10 +14341,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
         <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -14261,7 +14352,7 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4">
         <v>26.9815386</v>
@@ -14272,7 +14363,7 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5">
         <v>14.0067</v>
@@ -14283,7 +14374,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6" t="b">
         <v>0</v>
@@ -14291,7 +14382,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -14338,7 +14429,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="B11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -14385,7 +14476,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -14402,7 +14493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:11">
       <c r="A17">
         <v>1</v>
       </c>
@@ -14416,7 +14507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:11">
       <c r="A18">
         <v>1</v>
       </c>
@@ -14430,126 +14521,99 @@
         <v>4.68</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:11">
       <c r="A19">
         <v>1</v>
       </c>
       <c r="B19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20">
+        <v>1</v>
+      </c>
+      <c r="B20" t="s">
         <v>24</v>
       </c>
-      <c r="C19" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20">
-        <v>1</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>25</v>
       </c>
-      <c r="C20">
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21">
+        <v>1</v>
+      </c>
+      <c r="B21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:11">
+      <c r="A22">
+        <v>1</v>
+      </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C22" t="s">
-        <v>27</v>
-      </c>
-      <c r="D22" t="s">
         <v>28</v>
       </c>
-      <c r="E22" t="s">
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23">
+        <v>1</v>
+      </c>
+      <c r="B23" t="s">
         <v>29</v>
       </c>
-      <c r="F22" t="s">
+      <c r="C23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="B25" t="s">
         <v>30</v>
       </c>
-      <c r="G22" t="s">
+      <c r="C25" t="s">
         <v>31</v>
       </c>
-      <c r="H22" t="s">
+      <c r="D25" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="B23">
-        <v>0</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="E25" t="s">
         <v>33</v>
       </c>
-      <c r="D23">
-        <v>5</v>
-      </c>
-      <c r="E23">
-        <v>0</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23">
-        <v>0</v>
-      </c>
-      <c r="H23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="B24">
-        <v>1</v>
-      </c>
-      <c r="C24" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24">
-        <v>5</v>
-      </c>
-      <c r="E24">
-        <v>0</v>
-      </c>
-      <c r="F24">
-        <v>0</v>
-      </c>
-      <c r="G24">
-        <v>0</v>
-      </c>
-      <c r="H24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="B25">
-        <v>2</v>
-      </c>
-      <c r="C25" t="s">
-        <v>33</v>
-      </c>
-      <c r="D25">
-        <v>5</v>
-      </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-      <c r="G25">
-        <v>0</v>
-      </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
+      <c r="F25" t="s">
+        <v>34</v>
+      </c>
+      <c r="G25" t="s">
+        <v>35</v>
+      </c>
+      <c r="H25" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" t="s">
+        <v>37</v>
+      </c>
+      <c r="J25" t="s">
+        <v>38</v>
+      </c>
+      <c r="K25" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
       <c r="B26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C26" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D26">
         <v>5</v>
@@ -14566,13 +14630,22 @@
       <c r="H26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:8">
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
       <c r="B27">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D27">
         <v>5</v>
@@ -14589,13 +14662,22 @@
       <c r="H27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:8">
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
       <c r="B28">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D28">
         <v>5</v>
@@ -14612,13 +14694,22 @@
       <c r="H28">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:8">
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
       <c r="B29">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D29">
         <v>5</v>
@@ -14635,13 +14726,22 @@
       <c r="H29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:8">
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
       <c r="B30">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D30">
         <v>5</v>
@@ -14658,13 +14758,22 @@
       <c r="H30">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:8">
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
       <c r="B31">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D31">
         <v>5</v>
@@ -14681,13 +14790,22 @@
       <c r="H31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:8">
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
       <c r="B32">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C32" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D32">
         <v>5</v>
@@ -14704,13 +14822,22 @@
       <c r="H32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="2:8">
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11">
       <c r="B33">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C33" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -14727,13 +14854,22 @@
       <c r="H33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="2:8">
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11">
       <c r="B34">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C34" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D34">
         <v>5</v>
@@ -14748,6 +14884,111 @@
         <v>0</v>
       </c>
       <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <v>0</v>
+      </c>
+      <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:11">
+      <c r="B35">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35">
+        <v>5</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35">
+        <v>0</v>
+      </c>
+      <c r="I35">
+        <v>0</v>
+      </c>
+      <c r="J35">
+        <v>0</v>
+      </c>
+      <c r="K35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:11">
+      <c r="B36">
+        <v>10</v>
+      </c>
+      <c r="C36" t="s">
+        <v>40</v>
+      </c>
+      <c r="D36">
+        <v>5</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:11">
+      <c r="B37">
+        <v>11</v>
+      </c>
+      <c r="C37" t="s">
+        <v>40</v>
+      </c>
+      <c r="D37">
+        <v>5</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
         <v>0</v>
       </c>
     </row>
@@ -14763,27 +15004,27 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="B1" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="B2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -15069,972 +15310,1378 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:AK56"/>
+  <dimension ref="A2:AK94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C3">
         <v>7.2</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:3">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+        <v>49</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C5">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12">
+        <v>1</v>
+      </c>
+      <c r="B12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9">
-        <v>1</v>
-      </c>
-      <c r="B9" t="s">
+    <row r="13" spans="1:3">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14">
+        <v>1</v>
+      </c>
+      <c r="B14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="B15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16">
+        <v>1</v>
+      </c>
+      <c r="B16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19">
+        <v>1</v>
+      </c>
+      <c r="B19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20">
+        <v>1</v>
+      </c>
+      <c r="B20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" t="b">
+        <v>0</v>
+      </c>
+      <c r="D20" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21">
+        <v>1</v>
+      </c>
+      <c r="B21" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22">
+        <v>1</v>
+      </c>
+      <c r="B22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" t="s">
+        <v>73</v>
+      </c>
+      <c r="F22" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23">
+        <v>1</v>
+      </c>
+      <c r="B23" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" t="s">
+        <v>75</v>
+      </c>
+      <c r="D23" t="s">
+        <v>76</v>
+      </c>
+      <c r="E23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F23" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
+      <c r="A24">
+        <v>1</v>
+      </c>
+      <c r="B24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
+      <c r="A25">
+        <v>1</v>
+      </c>
+      <c r="B25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" t="s">
+        <v>81</v>
+      </c>
+      <c r="E25" t="s">
+        <v>82</v>
+      </c>
+      <c r="F25" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
+      <c r="A26">
+        <v>1</v>
+      </c>
+      <c r="B26" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>0.92</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
+      <c r="A27">
+        <v>1</v>
+      </c>
+      <c r="B27" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
+      <c r="A28">
+        <v>1</v>
+      </c>
+      <c r="B28" t="s">
+        <v>86</v>
+      </c>
+      <c r="C28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
+      <c r="A29">
+        <v>1</v>
+      </c>
+      <c r="B29" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
+      <c r="A30">
+        <v>1</v>
+      </c>
+      <c r="B30" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
+      <c r="A31">
+        <v>1</v>
+      </c>
+      <c r="B31" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
+      <c r="A32">
+        <v>1</v>
+      </c>
+      <c r="B32" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="1:37">
+      <c r="A33">
+        <v>1</v>
+      </c>
+      <c r="B33" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:37">
+      <c r="A34">
+        <v>1</v>
+      </c>
+      <c r="B34" t="s">
+        <v>95</v>
+      </c>
+      <c r="C34">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:37">
+      <c r="A35">
+        <v>1</v>
+      </c>
+      <c r="B35" t="s">
+        <v>96</v>
+      </c>
+      <c r="C35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="1:37">
+      <c r="A36">
+        <v>1</v>
+      </c>
+      <c r="B36" t="s">
+        <v>97</v>
+      </c>
+      <c r="C36">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:37">
+      <c r="A37">
+        <v>1</v>
+      </c>
+      <c r="B37" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:37">
+      <c r="A38">
+        <v>1</v>
+      </c>
+      <c r="B38" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="39" spans="1:37">
+      <c r="A39">
+        <v>1</v>
+      </c>
+      <c r="B39" t="s">
+        <v>100</v>
+      </c>
+      <c r="C39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:37">
+      <c r="A40">
+        <v>1</v>
+      </c>
+      <c r="B40" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="41" spans="1:37">
+      <c r="A41">
+        <v>1</v>
+      </c>
+      <c r="B41" t="s">
+        <v>103</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:37">
+      <c r="A42">
+        <v>1</v>
+      </c>
+      <c r="B42" t="s">
+        <v>104</v>
+      </c>
+      <c r="C42" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="43" spans="1:37">
+      <c r="A43">
+        <v>1</v>
+      </c>
+      <c r="B43" t="s">
+        <v>105</v>
+      </c>
+      <c r="C43">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="44" spans="1:37">
+      <c r="D44" t="s">
+        <v>106</v>
+      </c>
+      <c r="E44" t="s">
+        <v>107</v>
+      </c>
+      <c r="F44" t="s">
+        <v>108</v>
+      </c>
+      <c r="G44" t="s">
+        <v>109</v>
+      </c>
+      <c r="H44" t="s">
+        <v>108</v>
+      </c>
+      <c r="I44" t="s">
+        <v>110</v>
+      </c>
+      <c r="J44" t="s">
+        <v>111</v>
+      </c>
+      <c r="K44" t="s">
+        <v>112</v>
+      </c>
+      <c r="L44" t="s">
+        <v>107</v>
+      </c>
+      <c r="M44" t="s">
+        <v>110</v>
+      </c>
+      <c r="N44" t="s">
+        <v>113</v>
+      </c>
+      <c r="O44" t="s">
+        <v>109</v>
+      </c>
+      <c r="P44" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>115</v>
+      </c>
+      <c r="R44" t="s">
+        <v>108</v>
+      </c>
+      <c r="S44" t="s">
+        <v>112</v>
+      </c>
+      <c r="T44" t="s">
+        <v>113</v>
+      </c>
+      <c r="U44" t="s">
+        <v>109</v>
+      </c>
+      <c r="V44" t="s">
+        <v>114</v>
+      </c>
+      <c r="W44" t="s">
+        <v>116</v>
+      </c>
+      <c r="X44" t="s">
+        <v>117</v>
+      </c>
+      <c r="Y44" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z44" t="s">
+        <v>114</v>
+      </c>
+      <c r="AA44" t="s">
+        <v>111</v>
+      </c>
+      <c r="AB44" t="s">
+        <v>117</v>
+      </c>
+      <c r="AC44" t="s">
+        <v>112</v>
+      </c>
+      <c r="AD44" t="s">
+        <v>115</v>
+      </c>
+      <c r="AE44" t="s">
+        <v>113</v>
+      </c>
+      <c r="AF44" t="s">
+        <v>118</v>
+      </c>
+      <c r="AG44" t="s">
+        <v>112</v>
+      </c>
+      <c r="AH44" t="s">
+        <v>114</v>
+      </c>
+      <c r="AI44" t="s">
+        <v>119</v>
+      </c>
+      <c r="AJ44" t="s">
+        <v>108</v>
+      </c>
+      <c r="AK44" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="45" spans="1:37">
+      <c r="A45">
+        <v>1</v>
+      </c>
+      <c r="C45">
+        <v>2.668224269059857</v>
+      </c>
+      <c r="D45">
+        <v>-1.5405</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:37">
+      <c r="A46">
+        <v>1</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>3.081</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:37">
+      <c r="A47">
+        <v>1</v>
+      </c>
+      <c r="C47">
+        <v>0</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>5.030999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49">
+        <v>1</v>
+      </c>
+      <c r="B49" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50">
+        <v>1</v>
+      </c>
+      <c r="B50" t="s">
         <v>48</v>
       </c>
-      <c r="C9" t="b">
-        <v>0</v>
-      </c>
-      <c r="D9" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" t="b">
-        <v>0</v>
-      </c>
-      <c r="F9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C50">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51">
+        <v>1</v>
+      </c>
+      <c r="B51" t="s">
         <v>49</v>
       </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10">
-        <v>1</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C51" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52">
+        <v>1</v>
+      </c>
+      <c r="B52" t="s">
         <v>50</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C52">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53">
+        <v>1</v>
+      </c>
+      <c r="B53" t="s">
         <v>51</v>
       </c>
-      <c r="D11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="A12">
-        <v>1</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54">
+        <v>1</v>
+      </c>
+      <c r="B54" t="s">
         <v>52</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C54">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55">
+        <v>1</v>
+      </c>
+      <c r="B55" t="s">
         <v>53</v>
       </c>
-      <c r="D12" t="s">
+      <c r="C55" t="s">
         <v>54</v>
       </c>
-      <c r="E12" t="s">
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56">
+        <v>1</v>
+      </c>
+      <c r="B56" t="s">
         <v>55</v>
       </c>
-      <c r="F12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
-      <c r="A13">
-        <v>1</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C56" t="s">
         <v>56</v>
       </c>
-      <c r="C13" t="s">
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57">
+        <v>1</v>
+      </c>
+      <c r="B57" t="s">
         <v>57</v>
       </c>
-      <c r="D13" t="s">
-        <v>57</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="C57" t="s">
         <v>58</v>
       </c>
-      <c r="F13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="A14">
-        <v>1</v>
-      </c>
-      <c r="B14" t="s">
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58">
+        <v>1</v>
+      </c>
+      <c r="B58" t="s">
         <v>59</v>
       </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-      <c r="D14">
-        <v>0.92</v>
-      </c>
-      <c r="E14">
-        <v>1</v>
-      </c>
-      <c r="F14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
-      <c r="A15">
-        <v>1</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59">
+        <v>1</v>
+      </c>
+      <c r="B59" t="s">
         <v>60</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C59">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60">
+        <v>1</v>
+      </c>
+      <c r="B60" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="16" spans="1:14">
-      <c r="A16">
-        <v>1</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="C60" t="s">
         <v>62</v>
       </c>
-      <c r="C16" t="s">
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61">
+        <v>1</v>
+      </c>
+      <c r="B61" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="17" spans="1:37">
-      <c r="A17">
-        <v>1</v>
-      </c>
-      <c r="B17" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="C61">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62">
+        <v>1</v>
+      </c>
+      <c r="B62" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="18" spans="1:37">
-      <c r="A18">
-        <v>1</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="C62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63">
+        <v>1</v>
+      </c>
+      <c r="B63" t="s">
         <v>65</v>
       </c>
-      <c r="C18">
+      <c r="C63" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64">
+        <v>1</v>
+      </c>
+      <c r="B64" t="s">
+        <v>66</v>
+      </c>
+      <c r="C64">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14">
+      <c r="A65">
+        <v>1</v>
+      </c>
+      <c r="B65" t="s">
+        <v>67</v>
+      </c>
+      <c r="C65">
+        <v>0</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14">
+      <c r="A66">
+        <v>1</v>
+      </c>
+      <c r="B66" t="s">
+        <v>68</v>
+      </c>
+      <c r="C66" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14">
+      <c r="A67">
+        <v>1</v>
+      </c>
+      <c r="B67" t="s">
+        <v>70</v>
+      </c>
+      <c r="C67" t="b">
+        <v>0</v>
+      </c>
+      <c r="D67" t="b">
+        <v>0</v>
+      </c>
+      <c r="E67" t="b">
+        <v>1</v>
+      </c>
+      <c r="F67" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14">
+      <c r="A68">
+        <v>1</v>
+      </c>
+      <c r="B68" t="s">
+        <v>71</v>
+      </c>
+      <c r="C68">
+        <v>0</v>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68">
+        <v>0</v>
+      </c>
+      <c r="H68">
+        <v>1</v>
+      </c>
+      <c r="I68">
+        <v>0</v>
+      </c>
+      <c r="J68">
+        <v>0</v>
+      </c>
+      <c r="K68">
+        <v>1</v>
+      </c>
+      <c r="L68">
+        <v>0</v>
+      </c>
+      <c r="M68">
+        <v>0</v>
+      </c>
+      <c r="N68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14">
+      <c r="A69">
+        <v>1</v>
+      </c>
+      <c r="B69" t="s">
+        <v>72</v>
+      </c>
+      <c r="C69" t="s">
+        <v>73</v>
+      </c>
+      <c r="D69" t="s">
+        <v>73</v>
+      </c>
+      <c r="E69" t="s">
+        <v>73</v>
+      </c>
+      <c r="F69" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14">
+      <c r="A70">
+        <v>1</v>
+      </c>
+      <c r="B70" t="s">
+        <v>74</v>
+      </c>
+      <c r="C70" t="s">
+        <v>75</v>
+      </c>
+      <c r="D70" t="s">
+        <v>77</v>
+      </c>
+      <c r="E70" t="s">
+        <v>76</v>
+      </c>
+      <c r="F70" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
+      <c r="A71">
+        <v>1</v>
+      </c>
+      <c r="B71" t="s">
+        <v>78</v>
+      </c>
+      <c r="C71" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
+      <c r="A72">
+        <v>1</v>
+      </c>
+      <c r="B72" t="s">
+        <v>80</v>
+      </c>
+      <c r="C72" t="s">
+        <v>81</v>
+      </c>
+      <c r="D72" t="s">
+        <v>81</v>
+      </c>
+      <c r="E72" t="s">
+        <v>81</v>
+      </c>
+      <c r="F72" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
+      <c r="A73">
+        <v>1</v>
+      </c>
+      <c r="B73" t="s">
+        <v>83</v>
+      </c>
+      <c r="C73">
+        <v>1</v>
+      </c>
+      <c r="D73">
+        <v>0.24</v>
+      </c>
+      <c r="E73">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
+      <c r="A74">
+        <v>1</v>
+      </c>
+      <c r="B74" t="s">
+        <v>84</v>
+      </c>
+      <c r="C74" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
+      <c r="A75">
+        <v>1</v>
+      </c>
+      <c r="B75" t="s">
+        <v>86</v>
+      </c>
+      <c r="C75" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
+      <c r="A76">
+        <v>1</v>
+      </c>
+      <c r="B76" t="s">
+        <v>88</v>
+      </c>
+      <c r="C76" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14">
+      <c r="A77">
+        <v>1</v>
+      </c>
+      <c r="B77" t="s">
+        <v>90</v>
+      </c>
+      <c r="C77" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14">
+      <c r="A78">
+        <v>1</v>
+      </c>
+      <c r="B78" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14">
+      <c r="A79">
+        <v>1</v>
+      </c>
+      <c r="B79" t="s">
+        <v>93</v>
+      </c>
+      <c r="C79">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14">
+      <c r="A80">
+        <v>1</v>
+      </c>
+      <c r="B80" t="s">
+        <v>30</v>
+      </c>
+      <c r="C80" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="81" spans="1:37">
+      <c r="A81">
+        <v>1</v>
+      </c>
+      <c r="B81" t="s">
+        <v>95</v>
+      </c>
+      <c r="C81">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:37">
-      <c r="A19">
-        <v>1</v>
-      </c>
-      <c r="B19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C19">
+    <row r="82" spans="1:37">
+      <c r="A82">
+        <v>1</v>
+      </c>
+      <c r="B82" t="s">
+        <v>96</v>
+      </c>
+      <c r="C82">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:37">
-      <c r="A20">
-        <v>1</v>
-      </c>
-      <c r="B20" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20">
+    <row r="83" spans="1:37">
+      <c r="A83">
+        <v>1</v>
+      </c>
+      <c r="B83" t="s">
+        <v>97</v>
+      </c>
+      <c r="C83">
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:37">
-      <c r="A21">
-        <v>1</v>
-      </c>
-      <c r="B21" t="s">
-        <v>68</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:37">
-      <c r="A22">
-        <v>1</v>
-      </c>
-      <c r="B22" t="s">
-        <v>69</v>
-      </c>
-      <c r="C22" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="1:37">
-      <c r="A23">
-        <v>1</v>
-      </c>
-      <c r="B23" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:37">
-      <c r="A24">
-        <v>1</v>
-      </c>
-      <c r="B24" t="s">
-        <v>72</v>
-      </c>
-      <c r="C24" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="25" spans="1:37">
-      <c r="D25" t="s">
-        <v>73</v>
-      </c>
-      <c r="E25" t="s">
-        <v>74</v>
-      </c>
-      <c r="F25" t="s">
-        <v>75</v>
-      </c>
-      <c r="G25" t="s">
-        <v>76</v>
-      </c>
-      <c r="H25" t="s">
-        <v>75</v>
-      </c>
-      <c r="I25" t="s">
-        <v>77</v>
-      </c>
-      <c r="J25" t="s">
-        <v>78</v>
-      </c>
-      <c r="K25" t="s">
-        <v>79</v>
-      </c>
-      <c r="L25" t="s">
-        <v>74</v>
-      </c>
-      <c r="M25" t="s">
-        <v>77</v>
-      </c>
-      <c r="N25" t="s">
-        <v>80</v>
-      </c>
-      <c r="O25" t="s">
-        <v>76</v>
-      </c>
-      <c r="P25" t="s">
+    <row r="84" spans="1:37">
+      <c r="A84">
+        <v>1</v>
+      </c>
+      <c r="B84" t="s">
+        <v>98</v>
+      </c>
+      <c r="C84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:37">
+      <c r="A85">
+        <v>1</v>
+      </c>
+      <c r="B85" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="86" spans="1:37">
+      <c r="A86">
+        <v>1</v>
+      </c>
+      <c r="B86" t="s">
+        <v>100</v>
+      </c>
+      <c r="C86" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:37">
+      <c r="A87">
+        <v>1</v>
+      </c>
+      <c r="B87" t="s">
+        <v>101</v>
+      </c>
+      <c r="C87" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="88" spans="1:37">
+      <c r="A88">
+        <v>1</v>
+      </c>
+      <c r="B88" t="s">
+        <v>103</v>
+      </c>
+      <c r="C88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:37">
+      <c r="A89">
+        <v>1</v>
+      </c>
+      <c r="B89" t="s">
+        <v>104</v>
+      </c>
+      <c r="C89" t="s">
         <v>81</v>
       </c>
-      <c r="Q25" t="s">
-        <v>82</v>
-      </c>
-      <c r="R25" t="s">
-        <v>75</v>
-      </c>
-      <c r="S25" t="s">
-        <v>79</v>
-      </c>
-      <c r="T25" t="s">
-        <v>80</v>
-      </c>
-      <c r="U25" t="s">
-        <v>76</v>
-      </c>
-      <c r="V25" t="s">
-        <v>81</v>
-      </c>
-      <c r="W25" t="s">
-        <v>83</v>
-      </c>
-      <c r="X25" t="s">
-        <v>84</v>
-      </c>
-      <c r="Y25" t="s">
-        <v>79</v>
-      </c>
-      <c r="Z25" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA25" t="s">
-        <v>78</v>
-      </c>
-      <c r="AB25" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC25" t="s">
-        <v>79</v>
-      </c>
-      <c r="AD25" t="s">
-        <v>82</v>
-      </c>
-      <c r="AE25" t="s">
-        <v>80</v>
-      </c>
-      <c r="AF25" t="s">
-        <v>85</v>
-      </c>
-      <c r="AG25" t="s">
-        <v>79</v>
-      </c>
-      <c r="AH25" t="s">
-        <v>81</v>
-      </c>
-      <c r="AI25" t="s">
-        <v>86</v>
-      </c>
-      <c r="AJ25" t="s">
-        <v>75</v>
-      </c>
-      <c r="AK25" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="26" spans="1:37">
-      <c r="A26">
-        <v>1</v>
-      </c>
-      <c r="C26">
+    </row>
+    <row r="90" spans="1:37">
+      <c r="A90">
+        <v>1</v>
+      </c>
+      <c r="B90" t="s">
+        <v>105</v>
+      </c>
+      <c r="C90">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="91" spans="1:37">
+      <c r="D91" t="s">
+        <v>106</v>
+      </c>
+      <c r="E91" t="s">
+        <v>107</v>
+      </c>
+      <c r="F91" t="s">
+        <v>108</v>
+      </c>
+      <c r="G91" t="s">
+        <v>109</v>
+      </c>
+      <c r="H91" t="s">
+        <v>108</v>
+      </c>
+      <c r="I91" t="s">
+        <v>110</v>
+      </c>
+      <c r="J91" t="s">
+        <v>111</v>
+      </c>
+      <c r="K91" t="s">
+        <v>112</v>
+      </c>
+      <c r="L91" t="s">
+        <v>107</v>
+      </c>
+      <c r="M91" t="s">
+        <v>110</v>
+      </c>
+      <c r="N91" t="s">
+        <v>113</v>
+      </c>
+      <c r="O91" t="s">
+        <v>109</v>
+      </c>
+      <c r="P91" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q91" t="s">
+        <v>115</v>
+      </c>
+      <c r="R91" t="s">
+        <v>108</v>
+      </c>
+      <c r="S91" t="s">
+        <v>112</v>
+      </c>
+      <c r="T91" t="s">
+        <v>113</v>
+      </c>
+      <c r="U91" t="s">
+        <v>109</v>
+      </c>
+      <c r="V91" t="s">
+        <v>114</v>
+      </c>
+      <c r="W91" t="s">
+        <v>116</v>
+      </c>
+      <c r="X91" t="s">
+        <v>117</v>
+      </c>
+      <c r="Y91" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z91" t="s">
+        <v>114</v>
+      </c>
+      <c r="AA91" t="s">
+        <v>111</v>
+      </c>
+      <c r="AB91" t="s">
+        <v>117</v>
+      </c>
+      <c r="AC91" t="s">
+        <v>112</v>
+      </c>
+      <c r="AD91" t="s">
+        <v>115</v>
+      </c>
+      <c r="AE91" t="s">
+        <v>113</v>
+      </c>
+      <c r="AF91" t="s">
+        <v>118</v>
+      </c>
+      <c r="AG91" t="s">
+        <v>112</v>
+      </c>
+      <c r="AH91" t="s">
+        <v>114</v>
+      </c>
+      <c r="AI91" t="s">
+        <v>119</v>
+      </c>
+      <c r="AJ91" t="s">
+        <v>108</v>
+      </c>
+      <c r="AK91" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="92" spans="1:37">
+      <c r="A92">
+        <v>1</v>
+      </c>
+      <c r="C92">
         <v>2.668224269059857</v>
       </c>
-      <c r="D26">
+      <c r="D92">
         <v>-1.5405</v>
       </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:37">
-      <c r="A27">
-        <v>1</v>
-      </c>
-      <c r="C27">
-        <v>0</v>
-      </c>
-      <c r="D27">
+      <c r="E92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:37">
+      <c r="A93">
+        <v>1</v>
+      </c>
+      <c r="C93">
+        <v>0</v>
+      </c>
+      <c r="D93">
         <v>3.081</v>
       </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:37">
-      <c r="A28">
-        <v>1</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28">
-        <v>0</v>
-      </c>
-      <c r="E28">
-        <v>5.030999999999999</v>
-      </c>
-    </row>
-    <row r="30" spans="1:37">
-      <c r="A30">
-        <v>1</v>
-      </c>
-      <c r="B30" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="31" spans="1:37">
-      <c r="A31">
-        <v>1</v>
-      </c>
-      <c r="B31" t="s">
-        <v>41</v>
-      </c>
-      <c r="C31">
-        <v>7.2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:37">
-      <c r="A32">
-        <v>1</v>
-      </c>
-      <c r="B32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14">
-      <c r="A33">
-        <v>1</v>
-      </c>
-      <c r="B33" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14">
-      <c r="A34">
-        <v>1</v>
-      </c>
-      <c r="B34" t="s">
-        <v>44</v>
-      </c>
-      <c r="C34" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14">
-      <c r="A35">
-        <v>1</v>
-      </c>
-      <c r="B35" t="s">
-        <v>46</v>
-      </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14">
-      <c r="A36">
-        <v>1</v>
-      </c>
-      <c r="B36" t="s">
-        <v>47</v>
-      </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
-      <c r="D36">
-        <v>0</v>
-      </c>
-      <c r="E36">
-        <v>0</v>
-      </c>
-      <c r="F36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14">
-      <c r="A37">
-        <v>1</v>
-      </c>
-      <c r="B37" t="s">
-        <v>48</v>
-      </c>
-      <c r="C37" t="b">
-        <v>0</v>
-      </c>
-      <c r="D37" t="b">
-        <v>0</v>
-      </c>
-      <c r="E37" t="b">
-        <v>1</v>
-      </c>
-      <c r="F37" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14">
-      <c r="A38">
-        <v>1</v>
-      </c>
-      <c r="B38" t="s">
-        <v>49</v>
-      </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
-      <c r="D38">
-        <v>0</v>
-      </c>
-      <c r="E38">
-        <v>0</v>
-      </c>
-      <c r="F38">
-        <v>0</v>
-      </c>
-      <c r="G38">
-        <v>0</v>
-      </c>
-      <c r="H38">
-        <v>1</v>
-      </c>
-      <c r="I38">
-        <v>0</v>
-      </c>
-      <c r="J38">
-        <v>0</v>
-      </c>
-      <c r="K38">
-        <v>1</v>
-      </c>
-      <c r="L38">
-        <v>0</v>
-      </c>
-      <c r="M38">
-        <v>0</v>
-      </c>
-      <c r="N38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14">
-      <c r="A39">
-        <v>1</v>
-      </c>
-      <c r="B39" t="s">
-        <v>50</v>
-      </c>
-      <c r="C39" t="s">
-        <v>51</v>
-      </c>
-      <c r="D39" t="s">
-        <v>51</v>
-      </c>
-      <c r="E39" t="s">
-        <v>51</v>
-      </c>
-      <c r="F39" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14">
-      <c r="A40">
-        <v>1</v>
-      </c>
-      <c r="B40" t="s">
-        <v>52</v>
-      </c>
-      <c r="C40" t="s">
-        <v>53</v>
-      </c>
-      <c r="D40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E40" t="s">
-        <v>54</v>
-      </c>
-      <c r="F40" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14">
-      <c r="A41">
-        <v>1</v>
-      </c>
-      <c r="B41" t="s">
-        <v>56</v>
-      </c>
-      <c r="C41" t="s">
-        <v>57</v>
-      </c>
-      <c r="D41" t="s">
-        <v>57</v>
-      </c>
-      <c r="E41" t="s">
-        <v>57</v>
-      </c>
-      <c r="F41" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14">
-      <c r="A42">
-        <v>1</v>
-      </c>
-      <c r="B42" t="s">
-        <v>59</v>
-      </c>
-      <c r="C42">
-        <v>1</v>
-      </c>
-      <c r="D42">
-        <v>0.24</v>
-      </c>
-      <c r="E42">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="F42">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14">
-      <c r="A43">
-        <v>1</v>
-      </c>
-      <c r="B43" t="s">
-        <v>60</v>
-      </c>
-      <c r="C43" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14">
-      <c r="A44">
-        <v>1</v>
-      </c>
-      <c r="B44" t="s">
-        <v>62</v>
-      </c>
-      <c r="C44" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14">
-      <c r="A45">
-        <v>1</v>
-      </c>
-      <c r="B45" t="s">
-        <v>26</v>
-      </c>
-      <c r="C45" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="46" spans="1:14">
-      <c r="A46">
-        <v>1</v>
-      </c>
-      <c r="B46" t="s">
-        <v>65</v>
-      </c>
-      <c r="C46">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="47" spans="1:14">
-      <c r="A47">
-        <v>1</v>
-      </c>
-      <c r="B47" t="s">
-        <v>66</v>
-      </c>
-      <c r="C47">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="48" spans="1:14">
-      <c r="A48">
-        <v>1</v>
-      </c>
-      <c r="B48" t="s">
-        <v>67</v>
-      </c>
-      <c r="C48">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="49" spans="1:37">
-      <c r="A49">
-        <v>1</v>
-      </c>
-      <c r="B49" t="s">
-        <v>68</v>
-      </c>
-      <c r="C49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:37">
-      <c r="A50">
-        <v>1</v>
-      </c>
-      <c r="B50" t="s">
-        <v>69</v>
-      </c>
-      <c r="C50" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="51" spans="1:37">
-      <c r="A51">
-        <v>1</v>
-      </c>
-      <c r="B51" t="s">
-        <v>71</v>
-      </c>
-      <c r="C51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:37">
-      <c r="A52">
-        <v>1</v>
-      </c>
-      <c r="B52" t="s">
-        <v>72</v>
-      </c>
-      <c r="C52" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="53" spans="1:37">
-      <c r="D53" t="s">
-        <v>73</v>
-      </c>
-      <c r="E53" t="s">
-        <v>74</v>
-      </c>
-      <c r="F53" t="s">
-        <v>75</v>
-      </c>
-      <c r="G53" t="s">
-        <v>76</v>
-      </c>
-      <c r="H53" t="s">
-        <v>75</v>
-      </c>
-      <c r="I53" t="s">
-        <v>77</v>
-      </c>
-      <c r="J53" t="s">
-        <v>78</v>
-      </c>
-      <c r="K53" t="s">
-        <v>79</v>
-      </c>
-      <c r="L53" t="s">
-        <v>74</v>
-      </c>
-      <c r="M53" t="s">
-        <v>77</v>
-      </c>
-      <c r="N53" t="s">
-        <v>80</v>
-      </c>
-      <c r="O53" t="s">
-        <v>76</v>
-      </c>
-      <c r="P53" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q53" t="s">
-        <v>82</v>
-      </c>
-      <c r="R53" t="s">
-        <v>75</v>
-      </c>
-      <c r="S53" t="s">
-        <v>79</v>
-      </c>
-      <c r="T53" t="s">
-        <v>80</v>
-      </c>
-      <c r="U53" t="s">
-        <v>76</v>
-      </c>
-      <c r="V53" t="s">
-        <v>81</v>
-      </c>
-      <c r="W53" t="s">
-        <v>83</v>
-      </c>
-      <c r="X53" t="s">
-        <v>84</v>
-      </c>
-      <c r="Y53" t="s">
-        <v>79</v>
-      </c>
-      <c r="Z53" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA53" t="s">
-        <v>78</v>
-      </c>
-      <c r="AB53" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC53" t="s">
-        <v>79</v>
-      </c>
-      <c r="AD53" t="s">
-        <v>82</v>
-      </c>
-      <c r="AE53" t="s">
-        <v>80</v>
-      </c>
-      <c r="AF53" t="s">
-        <v>85</v>
-      </c>
-      <c r="AG53" t="s">
-        <v>79</v>
-      </c>
-      <c r="AH53" t="s">
-        <v>81</v>
-      </c>
-      <c r="AI53" t="s">
-        <v>86</v>
-      </c>
-      <c r="AJ53" t="s">
-        <v>75</v>
-      </c>
-      <c r="AK53" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="54" spans="1:37">
-      <c r="A54">
-        <v>1</v>
-      </c>
-      <c r="C54">
-        <v>2.668224269059857</v>
-      </c>
-      <c r="D54">
-        <v>-1.5405</v>
-      </c>
-      <c r="E54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:37">
-      <c r="A55">
-        <v>1</v>
-      </c>
-      <c r="C55">
-        <v>0</v>
-      </c>
-      <c r="D55">
-        <v>3.081</v>
-      </c>
-      <c r="E55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:37">
-      <c r="A56">
-        <v>1</v>
-      </c>
-      <c r="C56">
-        <v>0</v>
-      </c>
-      <c r="D56">
-        <v>0</v>
-      </c>
-      <c r="E56">
+      <c r="E93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:37">
+      <c r="A94">
+        <v>1</v>
+      </c>
+      <c r="C94">
+        <v>0</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94">
         <v>5.030999999999999</v>
       </c>
     </row>
@@ -16050,13 +16697,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -18885,13 +19532,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -21720,13 +22367,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -24555,13 +25202,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -27390,13 +28037,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4">

</xml_diff>